<commit_message>
edit components & main circuit
</commit_message>
<xml_diff>
--- a/hardware/pid-temperature-controller-hardware.xlsx
+++ b/hardware/pid-temperature-controller-hardware.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30110"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A4A83B5-06DC-4792-8362-966296D4ECCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{052C4E1F-53FD-4711-9922-A62D9336D4EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="28">
   <si>
     <t>Component</t>
   </si>
@@ -54,25 +54,37 @@
     <t>-</t>
   </si>
   <si>
-    <t>Temperature Sensor</t>
+    <t>Temperature Sensor [TH1]</t>
   </si>
   <si>
     <t>10K Waterproof NTC</t>
   </si>
   <si>
-    <t>Reference Resistor</t>
+    <t>Reference Resistor [R1]</t>
   </si>
   <si>
     <t>2660R</t>
   </si>
   <si>
-    <t>Power MOSFET</t>
+    <t>Gate Resistor [R2]</t>
+  </si>
+  <si>
+    <t>100R</t>
+  </si>
+  <si>
+    <t>Pull-Down Resistor [R3]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10K </t>
+  </si>
+  <si>
+    <t>Power MOSFET [Q1]</t>
   </si>
   <si>
     <t>IRLB8743</t>
   </si>
   <si>
-    <t>Heating Element</t>
+    <t>Heating Element [H1]</t>
   </si>
   <si>
     <t>12V/40W</t>
@@ -198,18 +210,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -532,152 +543,180 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="5" customFormat="1" ht="21" customHeight="1">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:4" s="4" customFormat="1" ht="21" customHeight="1">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8" t="s">
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="1" customFormat="1">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4">
-        <v>1</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" s="1" customFormat="1">
-      <c r="A3" s="2" t="s">
+      <c r="C2" s="3">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="1" customFormat="1">
-      <c r="A4" s="2" t="s">
+      <c r="C3" s="3">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="4">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" s="1" customFormat="1">
-      <c r="A5" s="2" t="s">
+      <c r="C4" s="3">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="4">
-        <v>1</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" s="1" customFormat="1">
-      <c r="A6" s="2" t="s">
+      <c r="C5" s="3">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="4">
-        <v>1</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="C6" s="3">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" s="1" customFormat="1">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="4">
-        <v>1</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" s="1" customFormat="1">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="4">
-        <v>1</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" s="1" customFormat="1">
-      <c r="A9" s="2" t="s">
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" s="1" customFormat="1">
-      <c r="A10" s="2" t="s">
+      <c r="C9" s="3">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="4">
-        <v>1</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="C10" s="3">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="3">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>